<commit_message>
add ProjectSearchDTO and test data for project search validation
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/dataCRM.xlsx
+++ b/src/test/resources/testdata/dataCRM.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRM_Automation_Testing\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4A8B01-3756-459A-9DD2-4CBAB8879234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB77827A-D53E-4B76-86DE-F9CC33CED849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Customers" sheetId="2" r:id="rId2"/>
     <sheet name="Projects" sheetId="4" r:id="rId3"/>
-    <sheet name="Tasks" sheetId="5" r:id="rId4"/>
+    <sheet name="Project_Search" sheetId="7" r:id="rId4"/>
+    <sheet name="Tasks" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="142">
   <si>
     <t>EMAIL</t>
   </si>
@@ -421,6 +422,39 @@
   </si>
   <si>
     <t>MauCT01.doc, HDTT.doc</t>
+  </si>
+  <si>
+    <t>KEYWORD_SEARCH</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>PROJECT_SEARCH</t>
+  </si>
+  <si>
+    <t>CUSTOMER_SEARCH</t>
+  </si>
+  <si>
+    <t>TAG_SEARCH</t>
+  </si>
+  <si>
+    <t>[AUTO_HT] project</t>
+  </si>
+  <si>
+    <t>[AUTO_HT] company</t>
+  </si>
+  <si>
+    <t>htest12</t>
+  </si>
+  <si>
+    <t>KEYWORD</t>
+  </si>
+  <si>
+    <t>CUSTOMER</t>
+  </si>
+  <si>
+    <t>TAG</t>
   </si>
 </sst>
 </file>
@@ -471,7 +505,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -492,6 +526,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -775,14 +812,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.53125" customWidth="1"/>
-    <col min="2" max="2" width="24.46484375" customWidth="1"/>
+    <col min="1" max="1" width="25.5546875" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -793,7 +830,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -804,7 +841,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -815,7 +852,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -840,23 +877,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.19921875" customWidth="1"/>
+    <col min="1" max="1" width="23.21875" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.19921875" customWidth="1"/>
-    <col min="5" max="5" width="11.1328125" customWidth="1"/>
-    <col min="6" max="6" width="13.46484375" customWidth="1"/>
-    <col min="7" max="7" width="11.53125" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="15.46484375" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="14.46484375" customWidth="1"/>
-    <col min="12" max="12" width="15.796875" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" customWidth="1"/>
+    <col min="12" max="12" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -894,7 +931,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>102</v>
       </c>
@@ -932,7 +969,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>102</v>
       </c>
@@ -979,28 +1016,33 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776F527C-2B5B-452D-B09B-948A7D4FA5C6}">
-  <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.46484375" customWidth="1"/>
-    <col min="2" max="2" width="18.796875" customWidth="1"/>
-    <col min="3" max="3" width="10.796875" customWidth="1"/>
-    <col min="4" max="4" width="13.1328125" customWidth="1"/>
-    <col min="5" max="5" width="11.53125" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.796875" customWidth="1"/>
-    <col min="8" max="8" width="22.1328125" customWidth="1"/>
-    <col min="9" max="9" width="16.86328125" customWidth="1"/>
-    <col min="10" max="10" width="15.796875" customWidth="1"/>
-    <col min="11" max="11" width="13.1328125" customWidth="1"/>
-    <col min="12" max="12" width="12.46484375" customWidth="1"/>
-    <col min="13" max="13" width="8.46484375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" customWidth="1"/>
+    <col min="11" max="11" width="13.109375" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="22.53125" customWidth="1"/>
+    <col min="16" max="16" width="22.5546875" customWidth="1"/>
+    <col min="17" max="17" width="10.44140625" customWidth="1"/>
+    <col min="18" max="18" width="17.21875" customWidth="1"/>
+    <col min="19" max="19" width="17" customWidth="1"/>
+    <col min="20" max="20" width="18.21875" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>61</v>
       </c>
@@ -1049,8 +1091,21 @@
       <c r="P1" s="4" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>103</v>
       </c>
@@ -1097,8 +1152,21 @@
       <c r="P2" s="7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="Q2" s="7"/>
+      <c r="R2" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="S2" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="T2" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>104</v>
       </c>
@@ -1145,8 +1213,9 @@
       <c r="P3" s="7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="Q3" s="7"/>
+    </row>
+    <row r="4" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>103</v>
       </c>
@@ -1191,8 +1260,9 @@
       <c r="P4" s="7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="Q4" s="7"/>
+    </row>
+    <row r="5" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>104</v>
       </c>
@@ -1237,6 +1307,7 @@
       <c r="P5" s="7" t="s">
         <v>41</v>
       </c>
+      <c r="Q5" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1246,32 +1317,77 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE7BF2E-42EA-4CC1-A3D3-4B565ADF5E90}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.5546875" customWidth="1"/>
+    <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C77C47-9B28-4F45-A10C-C7E9B32AD41D}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.06640625" customWidth="1"/>
+    <col min="1" max="1" width="17.109375" customWidth="1"/>
     <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.3984375" customWidth="1"/>
-    <col min="5" max="5" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.9296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.9296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.3984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.19921875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.21875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
@@ -1330,7 +1446,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="57" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>112</v>
       </c>
@@ -1384,7 +1500,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>113</v>
       </c>

</xml_diff>

<commit_message>
update data add/edit projects
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/dataCRM.xlsx
+++ b/src/test/resources/testdata/dataCRM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CRM_Automation_Testing\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB77827A-D53E-4B76-86DE-F9CC33CED849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6813A0EE-8DB5-48F9-A4A9-11DF5A417C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="138">
   <si>
     <t>EMAIL</t>
   </si>
@@ -424,21 +424,6 @@
     <t>MauCT01.doc, HDTT.doc</t>
   </si>
   <si>
-    <t>KEYWORD_SEARCH</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>PROJECT_SEARCH</t>
-  </si>
-  <si>
-    <t>CUSTOMER_SEARCH</t>
-  </si>
-  <si>
-    <t>TAG_SEARCH</t>
-  </si>
-  <si>
     <t>[AUTO_HT] project</t>
   </si>
   <si>
@@ -455,6 +440,9 @@
   </si>
   <si>
     <t>TAG</t>
+  </si>
+  <si>
+    <t>h</t>
   </si>
 </sst>
 </file>
@@ -812,14 +800,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
+    <col min="1" max="1" width="25.53125" customWidth="1"/>
+    <col min="2" max="2" width="24.46484375" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +818,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -841,7 +829,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -852,7 +840,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -877,23 +865,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="23.21875" customWidth="1"/>
+    <col min="1" max="1" width="23.19921875" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.19921875" customWidth="1"/>
+    <col min="5" max="5" width="11.1328125" customWidth="1"/>
+    <col min="6" max="6" width="13.46484375" customWidth="1"/>
+    <col min="7" max="7" width="11.53125" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="9" max="9" width="15.46484375" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="14.44140625" customWidth="1"/>
-    <col min="12" max="12" width="15.77734375" customWidth="1"/>
+    <col min="11" max="11" width="14.46484375" customWidth="1"/>
+    <col min="12" max="12" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -931,7 +919,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>102</v>
       </c>
@@ -969,7 +957,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>102</v>
       </c>
@@ -1016,33 +1004,28 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776F527C-2B5B-452D-B09B-948A7D4FA5C6}">
-  <dimension ref="A1:U5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="10.77734375" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="21.46484375" customWidth="1"/>
+    <col min="2" max="2" width="18.796875" customWidth="1"/>
+    <col min="3" max="3" width="10.796875" customWidth="1"/>
+    <col min="4" max="4" width="13.1328125" customWidth="1"/>
+    <col min="5" max="5" width="11.53125" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="22.109375" customWidth="1"/>
-    <col min="9" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="15.77734375" customWidth="1"/>
-    <col min="11" max="11" width="13.109375" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.796875" customWidth="1"/>
+    <col min="8" max="8" width="22.1328125" customWidth="1"/>
+    <col min="9" max="9" width="16.86328125" customWidth="1"/>
+    <col min="10" max="10" width="15.796875" customWidth="1"/>
+    <col min="11" max="11" width="13.1328125" customWidth="1"/>
+    <col min="12" max="12" width="12.46484375" customWidth="1"/>
+    <col min="13" max="13" width="8.46484375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.796875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="22.5546875" customWidth="1"/>
-    <col min="17" max="17" width="10.44140625" customWidth="1"/>
-    <col min="18" max="18" width="17.21875" customWidth="1"/>
-    <col min="19" max="19" width="17" customWidth="1"/>
-    <col min="20" max="20" width="18.21875" customWidth="1"/>
-    <col min="21" max="21" width="12.6640625" customWidth="1"/>
+    <col min="16" max="16" width="22.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>61</v>
       </c>
@@ -1091,21 +1074,8 @@
       <c r="P1" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:16" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" s="6" t="s">
         <v>103</v>
       </c>
@@ -1152,21 +1122,8 @@
       <c r="P2" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="S2" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="T2" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>104</v>
       </c>
@@ -1213,9 +1170,8 @@
       <c r="P3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Q3" s="7"/>
-    </row>
-    <row r="4" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>103</v>
       </c>
@@ -1260,9 +1216,8 @@
       <c r="P4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="7"/>
-    </row>
-    <row r="5" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
         <v>104</v>
       </c>
@@ -1307,7 +1262,6 @@
       <c r="P5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="Q5" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1319,40 +1273,40 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE7BF2E-42EA-4CC1-A3D3-4B565ADF5E90}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" customWidth="1"/>
-    <col min="2" max="2" width="23.77734375" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="1" max="1" width="19.53125" customWidth="1"/>
+    <col min="2" max="2" width="23.796875" customWidth="1"/>
+    <col min="3" max="3" width="21.46484375" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>137</v>
-      </c>
       <c r="D2" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1364,30 +1318,30 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C77C47-9B28-4F45-A10C-C7E9B32AD41D}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.1328125" customWidth="1"/>
     <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.46484375" customWidth="1"/>
+    <col min="5" max="5" width="9.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.86328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.53125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.19921875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.19921875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
@@ -1446,7 +1400,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="57" x14ac:dyDescent="0.45">
       <c r="A2" s="5" t="s">
         <v>112</v>
       </c>
@@ -1500,7 +1454,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>113</v>
       </c>

</xml_diff>